<commit_message>
se agregó voz y rango de edad
</commit_message>
<xml_diff>
--- a/data/Capacitacion/procesar/layoutPrueba.xlsx
+++ b/data/Capacitacion/procesar/layoutPrueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ikeasistencia0-my.sharepoint.com/personal/abolom_ikeasistencia_com/Documents/Documentos/1.-proyectos_ike/python/1.-Capacitacion_RH/2.-API.version_2.25022026/data/Capacitacion/procesar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="13_ncr:1_{16062AB9-70A9-4208-A972-0065B5D7523B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66132BC0-1B5C-412B-B89D-DD597549A028}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="114_{21CA807A-9DB4-40A2-9B0A-F90D8F72A0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FD8F9E9-999D-4931-A9C5-6040B2D91FEF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{580B104C-87EA-4B4E-8DBB-FEEBBC5B377A}"/>
   </bookViews>
@@ -57,10 +57,10 @@
     <t>+525539181750</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>399</t>
+    <t>4</t>
+  </si>
+  <si>
+    <t>377</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
se generan datos dinámicos
</commit_message>
<xml_diff>
--- a/data/Capacitacion/procesar/layoutPrueba.xlsx
+++ b/data/Capacitacion/procesar/layoutPrueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ikeasistencia0-my.sharepoint.com/personal/abolom_ikeasistencia_com/Documents/Documentos/1.-proyectos_ike/python/1.-Capacitacion_RH/2.-API.version_2.25022026/data/Capacitacion/procesar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="114_{21CA807A-9DB4-40A2-9B0A-F90D8F72A0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FD8F9E9-999D-4931-A9C5-6040B2D91FEF}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="114_{21CA807A-9DB4-40A2-9B0A-F90D8F72A0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34EED381-DA25-4A05-8D65-9D5B5F733B18}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{580B104C-87EA-4B4E-8DBB-FEEBBC5B377A}"/>
   </bookViews>
@@ -54,10 +54,10 @@
     <t>extension</t>
   </si>
   <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>+525539181750</t>
-  </si>
-  <si>
-    <t>4</t>
   </si>
   <si>
     <t>377</t>
@@ -482,10 +482,10 @@
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>11</v>

</xml_diff>